<commit_message>
Update weekly competition report
</commit_message>
<xml_diff>
--- a/reports/schedule_report.xlsx
+++ b/reports/schedule_report.xlsx
@@ -16,12 +16,12 @@
     <sheet name="疑似误抓取" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'日程总览'!$A$1:$P$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'日程总览'!$A$1:$P$44</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'比赛时间优先'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'报名截止提醒'!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'报名截止提醒'!$A$1:$P$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'结果公布提醒'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'可进日历'!$A$1:$P$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'待核实'!$A$1:$P$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'可进日历'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'待核实'!$A$1:$P$33</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'疑似误抓取'!$A$1:$P$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -3500,23 +3500,23 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>报名/报名截止</t>
+          <t>正式比赛</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>周期性/待核实</t>
+          <t>疑似误提取</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>以年度通知为准</t>
+          <t>2009-20</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>挑战杯中国大学生创业计划竞赛</t>
+          <t>挑战杯丨第十五届“挑战杯”新疆维吾尔自治区大学生创业计划竞赛圆满落幕</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3551,19 +3551,19 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>24</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
+          <t>https://www.tiaozhanbei.net/article/15858/</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
           <t>https://www.tiaozhanbei.net/</t>
         </is>
       </c>
-      <c r="N40" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tiaozhanbei.net/</t>
-        </is>
-      </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
           <t>否</t>
@@ -3571,14 +3571,14 @@
       </c>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>时间为周期性描述或需回源确认。</t>
+          <t>日期数值超出有效范围。</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>结果公布/获奖公示</t>
+          <t>报名/报名截止</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr"/>
@@ -3656,7 +3656,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>正式比赛</t>
+          <t>结果公布/获奖公示</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr"/>
@@ -3667,12 +3667,12 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>6月1日</t>
+          <t>以年度通知为准</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>竞赛章程（大挑）</t>
+          <t>挑战杯中国大学生创业计划竞赛</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3707,12 +3707,12 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>40</t>
         </is>
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>https://www.tiaozhanbei.net/rules</t>
+          <t>https://www.tiaozhanbei.net/</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3722,12 +3722,12 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>否</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>标题疑似导航/资讯/培训内容：章程。</t>
+          <t>时间为周期性描述或需回源确认。</t>
         </is>
       </c>
     </row>
@@ -3750,67 +3750,145 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
+          <t>竞赛章程（大挑）</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>创新创业类</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>P3 低优先级</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiaozhanbei.net/rules</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiaozhanbei.net/</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>标题疑似导航/资讯/培训内容：章程。</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>正式比赛</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>周期性/待核实</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>6月1日</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>竞赛章程（小挑）</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>创新创业类</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>P3 低优先级</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://www.tiaozhanbei.net/rules2</t>
         </is>
       </c>
-      <c r="N43" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>https://www.tiaozhanbei.net/</t>
         </is>
       </c>
-      <c r="O43" s="2" t="inlineStr">
+      <c r="O44" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="P43" s="2" t="inlineStr">
+      <c r="P44" s="2" t="inlineStr">
         <is>
           <t>标题疑似导航/资讯/培训内容：章程。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P43"/>
+  <autoFilter ref="A1:P44"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3936,14 +4014,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -3951,8 +4029,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
@@ -4039,86 +4117,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>报名/报名截止</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>具体日期</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026年9月10日</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>全国大学生数学建模竞赛</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>数学建模类</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>P1 优先关注</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mcm.edu.cn/index.moma</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mcm.edu.cn/index.moma</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4244,14 +4244,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -4259,8 +4259,8 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
-    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
@@ -4347,86 +4347,8 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>报名/报名截止</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-10</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>具体日期</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>2026年9月10日</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>全国大学生数学建模竞赛</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>数学建模类</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>P1 优先关注</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>46</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>48</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mcm.edu.cn/index.moma</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mcm.edu.cn/index.moma</t>
-        </is>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:P2"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4437,14 +4359,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
@@ -6781,23 +6703,23 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>报名/报名截止</t>
+          <t>正式比赛</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>周期性/待核实</t>
+          <t>疑似误提取</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>以年度通知为准</t>
+          <t>2009-20</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>挑战杯中国大学生创业计划竞赛</t>
+          <t>挑战杯丨第十五届“挑战杯”新疆维吾尔自治区大学生创业计划竞赛圆满落幕</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -6832,19 +6754,19 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>40</t>
+          <t>24</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
+          <t>https://www.tiaozhanbei.net/article/15858/</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
           <t>https://www.tiaozhanbei.net/</t>
         </is>
       </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.tiaozhanbei.net/</t>
-        </is>
-      </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
           <t>否</t>
@@ -6852,14 +6774,14 @@
       </c>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>时间为周期性描述或需回源确认。</t>
+          <t>日期数值超出有效范围。</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>结果公布/获奖公示</t>
+          <t>报名/报名截止</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr"/>
@@ -6934,8 +6856,86 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>结果公布/获奖公示</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>周期性/待核实</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>以年度通知为准</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>挑战杯中国大学生创业计划竞赛</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>创新创业类</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>P3 低优先级</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiaozhanbei.net/</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiaozhanbei.net/</t>
+        </is>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>时间为周期性描述或需回源确认。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P32"/>
+  <autoFilter ref="A1:P33"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>